<commit_message>
Rebuild AML, Dispute Resolution, and TPRM & Oversight tabs
Same pattern applied as Fraud: full SOW description per activity,
granular named sub-tasks, Req ID mapping to D3 vFinal (AML-XX, FD-XX,
TPA-XX, OS-XX), and sequentially numbered named deliverables per
activity. Deloitte Owner set to TBC pending staffing confirmation.
Existing manager edits (dates, notes, POCs) preserved where present.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Msiz5p6hoKmmUHZyLJTkqb
</commit_message>
<xml_diff>
--- a/Beem Visa Debit Transformation Phase Project Plan v3.xlsx
+++ b/Beem Visa Debit Transformation Phase Project Plan v3.xlsx
@@ -19,12 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="mmm\ d\,\ yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="mmm d, yyyy"/>
+    <numFmt numFmtId="165" formatCode="mmm d, yyyy"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,8 +130,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -191,6 +196,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F4F6FB"/>
         <bgColor rgb="00F4F6FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E2761"/>
+        <bgColor rgb="001E2761"/>
       </patternFill>
     </fill>
   </fills>
@@ -269,7 +280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -411,7 +422,7 @@
     <xf numFmtId="0" fontId="16" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -423,7 +434,7 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -438,11 +449,32 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="16" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1441,10 +1473,10 @@
           <t>DataVisor Product Owner (TBC) / Jesse Y.</t>
         </is>
       </c>
-      <c r="E15" s="51" t="n">
+      <c r="E15" s="63" t="n">
         <v>46286</v>
       </c>
-      <c r="F15" s="51" t="n">
+      <c r="F15" s="63" t="n">
         <v>46311</v>
       </c>
       <c r="G15" s="49" t="n"/>
@@ -1473,10 +1505,10 @@
           <t>Cynthia or Shikhar</t>
         </is>
       </c>
-      <c r="E16" s="55" t="n">
+      <c r="E16" s="64" t="n">
         <v>46286</v>
       </c>
-      <c r="F16" s="55" t="n">
+      <c r="F16" s="64" t="n">
         <v>46292</v>
       </c>
       <c r="G16" s="54" t="inlineStr">
@@ -1517,10 +1549,10 @@
           <t>Manoj</t>
         </is>
       </c>
-      <c r="E17" s="55" t="n">
+      <c r="E17" s="64" t="n">
         <v>46286</v>
       </c>
-      <c r="F17" s="55" t="n">
+      <c r="F17" s="64" t="n">
         <v>46290</v>
       </c>
       <c r="G17" s="54" t="n"/>
@@ -1557,10 +1589,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E18" s="55" t="n">
+      <c r="E18" s="64" t="n">
         <v>46293</v>
       </c>
-      <c r="F18" s="55" t="n">
+      <c r="F18" s="64" t="n">
         <v>46297</v>
       </c>
       <c r="G18" s="54" t="n"/>
@@ -1597,10 +1629,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E19" s="55" t="n">
+      <c r="E19" s="64" t="n">
         <v>46297</v>
       </c>
-      <c r="F19" s="55" t="n">
+      <c r="F19" s="64" t="n">
         <v>46302</v>
       </c>
       <c r="G19" s="54" t="n"/>
@@ -1637,10 +1669,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E20" s="55" t="n">
+      <c r="E20" s="64" t="n">
         <v>46302</v>
       </c>
-      <c r="F20" s="55" t="n">
+      <c r="F20" s="64" t="n">
         <v>46304</v>
       </c>
       <c r="G20" s="54" t="n"/>
@@ -1677,10 +1709,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E21" s="55" t="n">
+      <c r="E21" s="64" t="n">
         <v>46307</v>
       </c>
-      <c r="F21" s="55" t="n">
+      <c r="F21" s="64" t="n">
         <v>46311</v>
       </c>
       <c r="G21" s="54" t="n"/>
@@ -1715,10 +1747,10 @@
           <t>Shikhar / David / Cynthia (TBC); Manoj (technical)</t>
         </is>
       </c>
-      <c r="E22" s="51" t="n">
+      <c r="E22" s="63" t="n">
         <v>46314</v>
       </c>
-      <c r="F22" s="51" t="n">
+      <c r="F22" s="63" t="n">
         <v>46346</v>
       </c>
       <c r="G22" s="49" t="n"/>
@@ -1747,10 +1779,10 @@
           <t>Manoj</t>
         </is>
       </c>
-      <c r="E23" s="55" t="n">
+      <c r="E23" s="64" t="n">
         <v>46314</v>
       </c>
-      <c r="F23" s="55" t="n">
+      <c r="F23" s="64" t="n">
         <v>46318</v>
       </c>
       <c r="G23" s="54" t="n"/>
@@ -1787,10 +1819,10 @@
           <t>Shikhar/David/Cynthia</t>
         </is>
       </c>
-      <c r="E24" s="55" t="n">
+      <c r="E24" s="64" t="n">
         <v>46321</v>
       </c>
-      <c r="F24" s="55" t="n">
+      <c r="F24" s="64" t="n">
         <v>46325</v>
       </c>
       <c r="G24" s="54" t="n"/>
@@ -1827,10 +1859,10 @@
           <t>Shikhar/David/Cynthia</t>
         </is>
       </c>
-      <c r="E25" s="55" t="n">
+      <c r="E25" s="64" t="n">
         <v>46328</v>
       </c>
-      <c r="F25" s="55" t="n">
+      <c r="F25" s="64" t="n">
         <v>46335</v>
       </c>
       <c r="G25" s="54" t="n"/>
@@ -1867,10 +1899,10 @@
           <t>Shikhar/David/Cynthia</t>
         </is>
       </c>
-      <c r="E26" s="55" t="n">
+      <c r="E26" s="64" t="n">
         <v>46335</v>
       </c>
-      <c r="F26" s="55" t="n">
+      <c r="F26" s="64" t="n">
         <v>46339</v>
       </c>
       <c r="G26" s="54" t="n"/>
@@ -1907,10 +1939,10 @@
           <t>Shikhar/David/Cynthia</t>
         </is>
       </c>
-      <c r="E27" s="55" t="n">
+      <c r="E27" s="64" t="n">
         <v>46342</v>
       </c>
-      <c r="F27" s="55" t="n">
+      <c r="F27" s="64" t="n">
         <v>46346</v>
       </c>
       <c r="G27" s="54" t="n"/>
@@ -1945,10 +1977,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E28" s="51" t="n">
+      <c r="E28" s="63" t="n">
         <v>46335</v>
       </c>
-      <c r="F28" s="51" t="n">
+      <c r="F28" s="63" t="n">
         <v>46367</v>
       </c>
       <c r="G28" s="49" t="n"/>
@@ -1977,10 +2009,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E29" s="55" t="n">
+      <c r="E29" s="64" t="n">
         <v>46335</v>
       </c>
-      <c r="F29" s="55" t="n">
+      <c r="F29" s="64" t="n">
         <v>46339</v>
       </c>
       <c r="G29" s="54" t="n"/>
@@ -2017,10 +2049,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E30" s="55" t="n">
+      <c r="E30" s="64" t="n">
         <v>46342</v>
       </c>
-      <c r="F30" s="55" t="n">
+      <c r="F30" s="64" t="n">
         <v>46360</v>
       </c>
       <c r="G30" s="54" t="n"/>
@@ -2057,10 +2089,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E31" s="55" t="n">
+      <c r="E31" s="64" t="n">
         <v>46363</v>
       </c>
-      <c r="F31" s="55" t="n">
+      <c r="F31" s="64" t="n">
         <v>46367</v>
       </c>
       <c r="G31" s="54" t="n"/>
@@ -2095,10 +2127,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E32" s="51" t="n">
+      <c r="E32" s="63" t="n">
         <v>46349</v>
       </c>
-      <c r="F32" s="51" t="n">
+      <c r="F32" s="63" t="n">
         <v>46367</v>
       </c>
       <c r="G32" s="49" t="n"/>
@@ -2127,10 +2159,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E33" s="60" t="n">
+      <c r="E33" s="65" t="n">
         <v>46349</v>
       </c>
-      <c r="F33" s="60" t="n">
+      <c r="F33" s="65" t="n">
         <v>46351</v>
       </c>
       <c r="G33" s="56" t="n"/>
@@ -2167,10 +2199,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E34" s="60" t="n">
+      <c r="E34" s="65" t="n">
         <v>46351</v>
       </c>
-      <c r="F34" s="60" t="n">
+      <c r="F34" s="65" t="n">
         <v>46358</v>
       </c>
       <c r="G34" s="56" t="n"/>
@@ -2207,10 +2239,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E35" s="60" t="n">
+      <c r="E35" s="65" t="n">
         <v>46358</v>
       </c>
-      <c r="F35" s="60" t="n">
+      <c r="F35" s="65" t="n">
         <v>46360</v>
       </c>
       <c r="G35" s="56" t="n"/>
@@ -2247,10 +2279,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E36" s="60" t="n">
+      <c r="E36" s="65" t="n">
         <v>46360</v>
       </c>
-      <c r="F36" s="60" t="n">
+      <c r="F36" s="65" t="n">
         <v>46363</v>
       </c>
       <c r="G36" s="56" t="n"/>
@@ -2287,10 +2319,10 @@
           <t>Jesse Y.</t>
         </is>
       </c>
-      <c r="E37" s="60" t="n">
+      <c r="E37" s="65" t="n">
         <v>46363</v>
       </c>
-      <c r="F37" s="60" t="n">
+      <c r="F37" s="65" t="n">
         <v>46367</v>
       </c>
       <c r="G37" s="56" t="n"/>
@@ -2316,7 +2348,7 @@
       <c r="C38" s="56" t="n"/>
       <c r="D38" s="56" t="n"/>
       <c r="E38" s="59" t="n"/>
-      <c r="F38" s="60" t="n">
+      <c r="F38" s="65" t="n">
         <v>46367</v>
       </c>
       <c r="G38" s="56" t="n"/>
@@ -2339,17 +2371,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="19" min="1" max="1"/>
     <col width="52" customWidth="1" style="19" min="2" max="2"/>
     <col width="12" customWidth="1" style="19" min="3" max="3"/>
-    <col width="30" customWidth="1" style="19" min="4" max="4"/>
+    <col width="12.5" customWidth="1" style="19" min="4" max="4"/>
     <col width="13" customWidth="1" style="19" min="5" max="6"/>
+    <col width="13" customWidth="1" style="19" min="6" max="6"/>
     <col width="22" customWidth="1" style="19" min="7" max="7"/>
     <col width="12" customWidth="1" style="19" min="8" max="8"/>
-    <col width="68.77734375" customWidth="1" style="19" min="9" max="9"/>
+    <col width="13" customWidth="1" style="19" min="9" max="9"/>
+    <col width="68" customWidth="1" style="19" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.05" customHeight="1" s="19">
@@ -2363,587 +2397,856 @@
       <c r="A2" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="66" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Activity / Sub-Activity</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Point of Contact</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="B4" s="66" t="inlineStr">
+        <is>
+          <t>SOW Activity / Sub-Activity</t>
+        </is>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Deloitte Owner</t>
+        </is>
+      </c>
+      <c r="D4" s="66" t="inlineStr">
+        <is>
+          <t>Beem Point of Contact</t>
+        </is>
+      </c>
+      <c r="E4" s="66" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="66" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="66" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="66" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="I4" s="67" t="inlineStr">
+        <is>
+          <t>Req ID</t>
+        </is>
+      </c>
+      <c r="J4" s="68" t="inlineStr">
         <is>
           <t>Deliverables</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="55.2" customHeight="1" s="19">
-      <c r="A5" s="2" t="n">
+    <row r="5" ht="30" customHeight="1" s="19">
+      <c r="A5" s="48" t="n">
         <v>6</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Review the Current AML Process and Policy</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>Review and enhance the AML framework to support Visa Debit products and services, including policies, procedures, governance controls, sanctions screening requirements, investigation processes, regulatory, Sponsor Bank and Visa reporting obligations.</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="63" t="n">
         <v>46275</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="63" t="n">
         <v>46311</v>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I5" s="22" t="inlineStr">
-        <is>
-          <t>a. Policies, Procedures &amp; Governance Controls
-b. Sanctions Screening Requirements
-c. AML Investigation &amp; Case Management Processes
-d. Regulatory, Sponsor Bank &amp; Visa Reporting Requirements</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28.05" customHeight="1" s="19">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="G5" s="49" t="n"/>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="I5" s="52" t="n"/>
+      <c r="J5" s="57" t="n"/>
+    </row>
+    <row r="6" ht="24" customHeight="1" s="19">
+      <c r="A6" s="53" t="n"/>
+      <c r="B6" s="54" t="inlineStr">
         <is>
           <t>Collect and review current AML policy &amp; current AML alert, case, and regulatory reporting processes to identify potential gaps / changes</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="64" t="n">
         <v>46275</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="64" t="n">
         <v>46281</v>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="54" t="inlineStr">
         <is>
           <t>Due Thu Sept 10 EOD</t>
         </is>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="H6" s="53" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="I6" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Review and enhance the AML framework to support Visa Debit products and services, including policies, procedures, governance controls, sanctions screening requirements, investigation processes, regulatory, Sponsor Bank and Visa reporting obligations. </t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28.05" customHeight="1" s="19">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Conduct working sessions with AML team to validate and clarify understanding of AML framework (policies, governance controls, sanctions screening, investigation processes) and align on proposed gaps / changes</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="I6" s="42" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J6" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" s="19">
+      <c r="A7" s="53" t="n"/>
+      <c r="B7" s="54" t="inlineStr">
+        <is>
+          <t>Conduct working sessions with AML team to validate and clarify understanding of AML framework and align on proposed gaps / changes</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D7" s="54" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="64" t="n">
         <v>46279</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="64" t="n">
+        <v>46286</v>
+      </c>
+      <c r="G7" s="54" t="n"/>
+      <c r="H7" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I7" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J7" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" s="19">
+      <c r="A8" s="53" t="n"/>
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t>Draft enhanced AML policies, procedures &amp; governance controls</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E8" s="64" t="n">
+        <v>46286</v>
+      </c>
+      <c r="F8" s="64" t="n">
+        <v>46290</v>
+      </c>
+      <c r="G8" s="54" t="n"/>
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I8" s="59" t="inlineStr">
+        <is>
+          <t>AML-01</t>
+        </is>
+      </c>
+      <c r="J8" s="56" t="inlineStr">
+        <is>
+          <t>1. Enhanced AML Policies, Procedures &amp; Governance Controls (Visa Debit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" s="19">
+      <c r="A9" s="53" t="n"/>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>Draft sanctions screening process &amp; requirements</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E9" s="64" t="n">
+        <v>46290</v>
+      </c>
+      <c r="F9" s="64" t="n">
+        <v>46294</v>
+      </c>
+      <c r="G9" s="54" t="n"/>
+      <c r="H9" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I9" s="59" t="inlineStr">
+        <is>
+          <t>AML-03, AML-05</t>
+        </is>
+      </c>
+      <c r="J9" s="56" t="inlineStr">
+        <is>
+          <t>2. Sanctions Screening Process &amp; Requirements (OFAC SDN screening, true-match card/account disablement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1" s="19">
+      <c r="A10" s="53" t="n"/>
+      <c r="B10" s="54" t="inlineStr">
+        <is>
+          <t>Draft AML investigation &amp; case management process</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E10" s="64" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F10" s="64" t="n">
+        <v>46300</v>
+      </c>
+      <c r="G10" s="54" t="n"/>
+      <c r="H10" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I10" s="42" t="inlineStr">
+        <is>
+          <t>AML-01</t>
+        </is>
+      </c>
+      <c r="J10" s="56" t="inlineStr">
+        <is>
+          <t>3. AML Investigation &amp; Case Management Process</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" s="19">
+      <c r="A11" s="53" t="n"/>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>Draft regulatory, Sponsor Bank &amp; Visa reporting requirements (FINTRAC, ICICI)</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E11" s="64" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F11" s="64" t="n">
         <v>46304</v>
       </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I7" s="61" t="n"/>
-    </row>
-    <row r="8" ht="28.05" customHeight="1" s="19">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Draft enhanced AML framework (policies, governance controls, sanctions screening, investigation processes)</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="G11" s="54" t="n"/>
+      <c r="H11" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I11" s="42" t="inlineStr">
+        <is>
+          <t>AML-06, AML-07, AML-08</t>
+        </is>
+      </c>
+      <c r="J11" s="56" t="inlineStr">
+        <is>
+          <t>4. AML Regulatory &amp; Sponsor Bank Reporting Requirements (FINTRAC STR/EFT/LCT, ICICI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" s="19">
+      <c r="A12" s="53" t="n"/>
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>Review &amp; finalize with Beem stakeholders</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n">
-        <v>46279</v>
-      </c>
-      <c r="F8" s="7" t="n">
+      <c r="E12" s="64" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F12" s="64" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G12" s="54" t="n"/>
+      <c r="H12" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I12" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J12" s="56" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" s="19">
+      <c r="A13" s="48" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>Design, build and operationalize the AML monitoring framework for Visa Debit activity, including monitoring methodologies, monitoring rules, alert scenarios, testing, and production readiness activities.</t>
+        </is>
+      </c>
+      <c r="C13" s="49" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D13" s="49" t="inlineStr">
+        <is>
+          <t>Sandra M.; Navaera Relationship Owner (TBC)</t>
+        </is>
+      </c>
+      <c r="E13" s="63" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F13" s="63" t="n">
+        <v>46332</v>
+      </c>
+      <c r="G13" s="49" t="n"/>
+      <c r="H13" s="48" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I13" s="58" t="n"/>
+      <c r="J13" s="57" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1" s="19">
+      <c r="A14" s="53" t="n"/>
+      <c r="B14" s="54" t="inlineStr">
+        <is>
+          <t>Beem to introduce Deloitte to Navaera to discuss PCI-compliance workaround</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M. / Navaera Relationship Owner (TBC)</t>
+        </is>
+      </c>
+      <c r="E14" s="64" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F14" s="64" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G14" s="54" t="inlineStr">
+        <is>
+          <t>Kwaseem from Navaera to coordinate time</t>
+        </is>
+      </c>
+      <c r="H14" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I14" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J14" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="19">
+      <c r="A15" s="53" t="n"/>
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>Assess whether Navaera's workaround is sufficient; confirm build approach</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D15" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E15" s="64" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F15" s="64" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G15" s="54" t="n"/>
+      <c r="H15" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I15" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J15" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1" s="19">
+      <c r="A16" s="53" t="n"/>
+      <c r="B16" s="54" t="inlineStr">
+        <is>
+          <t>Draft AML monitoring methodology &amp; risk coverage approach</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E16" s="64" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F16" s="64" t="n">
         <v>46304</v>
       </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I8" s="61" t="n"/>
-    </row>
-    <row r="9" ht="28.05" customHeight="1" s="19">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="G16" s="54" t="n"/>
+      <c r="H16" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I16" s="42" t="inlineStr">
+        <is>
+          <t>AML-02</t>
+        </is>
+      </c>
+      <c r="J16" s="56" t="inlineStr">
+        <is>
+          <t>1. AML Monitoring Methodology &amp; Risk Coverage Approach</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1" s="19">
+      <c r="A17" s="53" t="n"/>
+      <c r="B17" s="54" t="inlineStr">
+        <is>
+          <t>Draft AML monitoring rules &amp; alert scenarios</t>
+        </is>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D17" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E17" s="64" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F17" s="64" t="n">
+        <v>46311</v>
+      </c>
+      <c r="G17" s="54" t="n"/>
+      <c r="H17" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I17" s="42" t="inlineStr">
+        <is>
+          <t>AML-02, AML-11</t>
+        </is>
+      </c>
+      <c r="J17" s="56" t="inlineStr">
+        <is>
+          <t>2. AML Monitoring Rules &amp; Alert Scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1" s="19">
+      <c r="A18" s="53" t="n"/>
+      <c r="B18" s="54" t="inlineStr">
+        <is>
+          <t>Conduct testing &amp; validation of AML monitoring rules</t>
+        </is>
+      </c>
+      <c r="C18" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D18" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E18" s="64" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F18" s="64" t="n">
+        <v>46320</v>
+      </c>
+      <c r="G18" s="54" t="n"/>
+      <c r="H18" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I18" s="59" t="inlineStr">
+        <is>
+          <t>AML-12</t>
+        </is>
+      </c>
+      <c r="J18" s="56" t="inlineStr">
+        <is>
+          <t>3. AML Monitoring Rules Testing &amp; Validation Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1" s="19">
+      <c r="A19" s="53" t="n"/>
+      <c r="B19" s="54" t="inlineStr">
+        <is>
+          <t>Complete production readiness &amp; operationalization activities</t>
+        </is>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D19" s="54" t="inlineStr">
+        <is>
+          <t>Sandra M.</t>
+        </is>
+      </c>
+      <c r="E19" s="64" t="n">
+        <v>46321</v>
+      </c>
+      <c r="F19" s="64" t="n">
+        <v>46325</v>
+      </c>
+      <c r="G19" s="54" t="n"/>
+      <c r="H19" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I19" s="59" t="inlineStr">
+        <is>
+          <t>AML-12, AML-13</t>
+        </is>
+      </c>
+      <c r="J19" s="56" t="inlineStr">
+        <is>
+          <t>4. AML Monitoring Production Readiness &amp; Operationalization Checklist</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1" s="19">
+      <c r="A20" s="53" t="n"/>
+      <c r="B20" s="54" t="inlineStr">
         <is>
           <t>Review &amp; finalize with Beem stakeholders</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="C20" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D20" s="54" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I9" s="62" t="n"/>
-    </row>
-    <row r="10" ht="55.2" customHeight="1" s="19">
-      <c r="A10" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Update the AML Monitoring Process</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Sandra M.; Navaera Relationship Owner (TBC)</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F10" s="4" t="n">
+      <c r="E20" s="64" t="n">
+        <v>46328</v>
+      </c>
+      <c r="F20" s="64" t="n">
         <v>46332</v>
       </c>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I10" s="22" t="inlineStr">
-        <is>
-          <t>a. Monitoring Methodology &amp; Risk Coverage
-b. Monitoring Rules &amp; Alert Scenarios
-c. Testing &amp; Validation Activities
-d. Production Readiness &amp; Operationalization Activities</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28.05" customHeight="1" s="19">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Beem to introduce Deloitte to Navaera to discuss PCI-compliance workaround</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Sandra M. / Navaera Relationship Owner (TBC)</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>46297</v>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>Kwaseem from Navaera to coordinate time</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I11" s="23" t="inlineStr">
-        <is>
-          <t>Design, build and operationalize the AML monitoring framework for Visa Debit activity, including monitoring methodologies, monitoring rules, alert scenarios, testing, and production readiness activities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28.05" customHeight="1" s="19">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Assess whether Navaera's workaround is sufficient; confirm build approach</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="G20" s="54" t="n"/>
+      <c r="H20" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I20" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J20" s="56" t="n"/>
+    </row>
+    <row r="21" ht="30" customHeight="1" s="19">
+      <c r="A21" s="58" t="n">
+        <v>8</v>
+      </c>
+      <c r="B21" s="57" t="inlineStr">
+        <is>
+          <t>Design and implement an internal AML reporting framework, including operational and analytics performance reports.</t>
+        </is>
+      </c>
+      <c r="C21" s="57" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D21" s="57" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F12" s="7" t="n">
-        <v>46297</v>
-      </c>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I12" s="61" t="n"/>
-    </row>
-    <row r="13" ht="28.05" customHeight="1" s="19">
-      <c r="A13" s="5" t="n"/>
-      <c r="B13" s="6" t="inlineStr">
-        <is>
-          <t>Design monitoring methodologies, monitoring rules &amp; alert scenarios</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="E21" s="69" t="n">
+        <v>46335</v>
+      </c>
+      <c r="F21" s="69" t="n">
+        <v>46353</v>
+      </c>
+      <c r="G21" s="57" t="n"/>
+      <c r="H21" s="58" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I21" s="58" t="n"/>
+      <c r="J21" s="57" t="n"/>
+    </row>
+    <row r="22" ht="24" customHeight="1" s="19">
+      <c r="A22" s="59" t="n"/>
+      <c r="B22" s="56" t="inlineStr">
+        <is>
+          <t>Collect current AML reports/dashboards &amp; reporting cadence/formats</t>
+        </is>
+      </c>
+      <c r="C22" s="56" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D22" s="56" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E13" s="7" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>46311</v>
-      </c>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I13" s="61" t="n"/>
-    </row>
-    <row r="14" ht="28.05" customHeight="1" s="19">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>Testing &amp; production readiness activities</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="E22" s="65" t="n">
+        <v>46335</v>
+      </c>
+      <c r="F22" s="65" t="n">
+        <v>46337</v>
+      </c>
+      <c r="G22" s="56" t="n"/>
+      <c r="H22" s="59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I22" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J22" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1" s="19">
+      <c r="A23" s="59" t="n"/>
+      <c r="B23" s="56" t="inlineStr">
+        <is>
+          <t>Draft internal AML reporting framework (operational &amp; analytics performance reports)</t>
+        </is>
+      </c>
+      <c r="C23" s="56" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D23" s="56" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E14" s="7" t="n">
-        <v>46314</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>46325</v>
-      </c>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I14" s="61" t="n"/>
-    </row>
-    <row r="15" ht="28.05" customHeight="1" s="19">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Review &amp; finalize with Beem stakeholders</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="E23" s="65" t="n">
+        <v>46338</v>
+      </c>
+      <c r="F23" s="65" t="n">
+        <v>46346</v>
+      </c>
+      <c r="G23" s="56" t="n"/>
+      <c r="H23" s="59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I23" s="59" t="inlineStr">
+        <is>
+          <t>AML-09, AML-10</t>
+        </is>
+      </c>
+      <c r="J23" s="56" t="inlineStr">
+        <is>
+          <t>1. Internal AML Reporting Framework (operational &amp; analytics performance reports)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1" s="19">
+      <c r="A24" s="59" t="n"/>
+      <c r="B24" s="56" t="inlineStr">
+        <is>
+          <t>Review &amp; finalize with stakeholders</t>
+        </is>
+      </c>
+      <c r="C24" s="56" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D24" s="56" t="inlineStr">
         <is>
           <t>Sandra M.</t>
         </is>
       </c>
-      <c r="E15" s="7" t="n">
-        <v>46328</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>46332</v>
-      </c>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I15" s="62" t="n"/>
-    </row>
-    <row r="16" ht="30" customHeight="1" s="19">
-      <c r="A16" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Update AML Reporting Process</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Sandra M.</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>46335</v>
-      </c>
-      <c r="F16" s="4" t="n">
+      <c r="E24" s="65" t="n">
+        <v>46349</v>
+      </c>
+      <c r="F24" s="65" t="n">
         <v>46353</v>
       </c>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I16" s="22" t="inlineStr">
-        <is>
-          <t>a. Internal AML Reporting Frameworks (operational &amp; analytics performance reports)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="28.05" customHeight="1" s="19">
-      <c r="A17" s="5" t="n"/>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Collect current AML reports/dashboards &amp; reporting cadence/formats</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Sandra M.</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>46335</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>46337</v>
-      </c>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I17" s="23" t="inlineStr">
-        <is>
-          <t>Design and implement an internal AML reporting framework, including operational and analytics performance reports.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="28.05" customHeight="1" s="19">
-      <c r="A18" s="5" t="n"/>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Draft internal AML reporting framework (operational &amp; analytics performance reports)</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Sandra M.</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>46338</v>
-      </c>
-      <c r="F18" s="7" t="n">
-        <v>46346</v>
-      </c>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I18" s="61" t="n"/>
-    </row>
-    <row r="19" ht="28.05" customHeight="1" s="19">
-      <c r="A19" s="5" t="n"/>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>Review &amp; finalize with stakeholders</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Sandra M.</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>46349</v>
-      </c>
-      <c r="F19" s="7" t="n">
+      <c r="G24" s="56" t="n"/>
+      <c r="H24" s="59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I24" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J24" s="56" t="n"/>
+    </row>
+    <row r="25" ht="24" customHeight="1" s="19">
+      <c r="A25" s="59" t="n"/>
+      <c r="B25" s="56" t="inlineStr">
+        <is>
+          <t>Completion of AML Transformation Activities</t>
+        </is>
+      </c>
+      <c r="C25" s="56" t="n"/>
+      <c r="D25" s="56" t="n"/>
+      <c r="E25" s="59" t="n"/>
+      <c r="F25" s="65" t="n">
         <v>46353</v>
       </c>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I19" s="62" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="n"/>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Completion of AML Transformation Activities</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="inlineStr">
-        <is>
-          <t>Milestone</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n">
-        <v>46353</v>
-      </c>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="8" t="n"/>
+      <c r="G25" s="56" t="n"/>
+      <c r="H25" s="59" t="n"/>
+      <c r="I25" s="59" t="n"/>
+      <c r="J25" s="56" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="I11:I15"/>
-    <mergeCell ref="I17:I19"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I6:I9"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2956,17 +3259,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="19" min="1" max="1"/>
     <col width="52" customWidth="1" style="19" min="2" max="2"/>
     <col width="12" customWidth="1" style="19" min="3" max="3"/>
-    <col width="30" customWidth="1" style="19" min="4" max="4"/>
+    <col width="12.5" customWidth="1" style="19" min="4" max="4"/>
     <col width="13" customWidth="1" style="19" min="5" max="6"/>
+    <col width="13" customWidth="1" style="19" min="6" max="6"/>
     <col width="22" customWidth="1" style="19" min="7" max="7"/>
     <col width="12" customWidth="1" style="19" min="8" max="8"/>
-    <col width="68.77734375" customWidth="1" style="19" min="9" max="9"/>
+    <col width="13" customWidth="1" style="19" min="9" max="9"/>
+    <col width="68" customWidth="1" style="19" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.05" customHeight="1" s="19">
@@ -2980,306 +3285,426 @@
       <c r="A2" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="66" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Activity / Sub-Activity</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Point of Contact</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="B4" s="66" t="inlineStr">
+        <is>
+          <t>SOW Activity / Sub-Activity</t>
+        </is>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Deloitte Owner</t>
+        </is>
+      </c>
+      <c r="D4" s="66" t="inlineStr">
+        <is>
+          <t>Beem Point of Contact</t>
+        </is>
+      </c>
+      <c r="E4" s="66" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="66" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="66" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="66" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="I4" s="67" t="inlineStr">
+        <is>
+          <t>Req ID</t>
+        </is>
+      </c>
+      <c r="J4" s="68" t="inlineStr">
         <is>
           <t>Deliverables</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1" s="19">
-      <c r="A5" s="2" t="n">
+    <row r="5" ht="30" customHeight="1" s="19">
+      <c r="A5" s="48" t="n">
         <v>9</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Build Target-state Dispute Management Process</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>Design and document the end-to-end dispute management lifecycle, including dispute intake, fraud or non-fraud determination, provisional credit issuance, chargeback submission (via Central 1), Visa dispute processing, and funds recovery activities. Deliver supporting procedures, process maps, and operational controls to support efficient dispute resolution and recovery operations.</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
         <is>
           <t>Loni B. (Non-fraud Disputes); Pattie L. (Fraudulent Disputes)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="63" t="n">
         <v>46279</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="63" t="n">
         <v>46311</v>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I5" s="27" t="inlineStr">
-        <is>
-          <t>a. Target-State Dispute Management Lifecycle Design
-b. Supporting Dispute Procedures, Process Maps &amp; Operational Controls</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28.05" customHeight="1" s="19">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>Design target-state dispute lifecycle (intake, fraud/non-fraud determination, provisional credit, chargeback via Central 1, Visa processing, funds recovery)</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="G5" s="49" t="n"/>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I5" s="52" t="n"/>
+      <c r="J5" s="57" t="n"/>
+    </row>
+    <row r="6" ht="24" customHeight="1" s="19">
+      <c r="A6" s="53" t="n"/>
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>Draft target-state dispute intake &amp; fraud/non-fraud determination process</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="inlineStr">
         <is>
           <t>Loni B. / Pattie L.</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="64" t="n">
         <v>46279</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="64" t="n">
+        <v>46287</v>
+      </c>
+      <c r="G6" s="54" t="n"/>
+      <c r="H6" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I6" s="42" t="inlineStr">
+        <is>
+          <t>FD-05, FD-06</t>
+        </is>
+      </c>
+      <c r="J6" s="56" t="inlineStr">
+        <is>
+          <t>1. Target-State Dispute Intake &amp; Fraud/Non-Fraud Determination Process</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" s="19">
+      <c r="A7" s="53" t="n"/>
+      <c r="B7" s="54" t="inlineStr">
+        <is>
+          <t>Draft target-state provisional credit, chargeback submission (Central 1) &amp; Visa dispute processing flow</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D7" s="54" t="inlineStr">
+        <is>
+          <t>Loni B. / Pattie L.</t>
+        </is>
+      </c>
+      <c r="E7" s="64" t="n">
+        <v>46287</v>
+      </c>
+      <c r="F7" s="64" t="n">
+        <v>46295</v>
+      </c>
+      <c r="G7" s="54" t="n"/>
+      <c r="H7" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I7" s="59" t="inlineStr">
+        <is>
+          <t>FD-09</t>
+        </is>
+      </c>
+      <c r="J7" s="56" t="inlineStr">
+        <is>
+          <t>2. Target-State Provisional Credit, Chargeback (Central 1) &amp; Visa Dispute Processing Flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" s="19">
+      <c r="A8" s="53" t="n"/>
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t>Draft target-state funds recovery process &amp; supporting procedures/process maps</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="inlineStr">
+        <is>
+          <t>Loni B. / Pattie L.</t>
+        </is>
+      </c>
+      <c r="E8" s="64" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F8" s="64" t="n">
         <v>46311</v>
       </c>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I6" s="28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Design and document the end-to-end dispute management lifecycle, including dispute intake, fraud or non-fraud determination, provisional credit issuance (see out of scope activity #1), chargeback submission (via Central 1), Visa dispute processing, and funds recovery activities. Deliver supporting procedures, process maps, and operational controls to support efficient dispute resolution and recovery operations. </t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1" s="19">
-      <c r="A7" s="2" t="n">
+      <c r="G8" s="54" t="n"/>
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I8" s="59" t="inlineStr">
+        <is>
+          <t>FD-10</t>
+        </is>
+      </c>
+      <c r="J8" s="56" t="inlineStr">
+        <is>
+          <t>3. Target-State Funds Recovery Process &amp; Supporting Procedures/Process Maps</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1" s="19">
+      <c r="A9" s="48" t="n">
         <v>10</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B9" s="49" t="inlineStr">
         <is>
           <t>Refine / Finalize Target-State Process</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="C9" s="49" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D9" s="49" t="inlineStr">
         <is>
           <t>Loni B. (Non-fraud Disputes); Pattie L. (Fraudulent Disputes)</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E9" s="63" t="n">
         <v>46307</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="F9" s="63" t="n">
         <v>46346</v>
       </c>
-      <c r="G7" s="3" t="n"/>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I7" s="61" t="n"/>
-    </row>
-    <row r="8" ht="30" customHeight="1" s="19">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="G9" s="49" t="n"/>
+      <c r="H9" s="48" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I9" s="58" t="n"/>
+      <c r="J9" s="57" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1" s="19">
+      <c r="A10" s="53" t="n"/>
+      <c r="B10" s="54" t="inlineStr">
         <is>
           <t>Collect and review current dispute policies/process (incl. Central 1) &amp; current dispute forms/templates/comms</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="inlineStr">
         <is>
           <t>Loni B. / Pattie L.</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E10" s="64" t="n">
         <v>46307</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F10" s="64" t="n">
         <v>46311</v>
       </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I8" s="61" t="n"/>
-    </row>
-    <row r="9" ht="28.05" customHeight="1" s="19">
-      <c r="A9" s="5" t="n"/>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Compare target-state design against Beem's current-state dispute process </t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="G10" s="54" t="n"/>
+      <c r="H10" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I10" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1" s="19">
+      <c r="A11" s="53" t="n"/>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>Compare target-state design against Beem's current-state dispute process</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D11" s="54" t="inlineStr">
         <is>
           <t>Loni B. / Pattie L.</t>
         </is>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E11" s="64" t="n">
         <v>46314</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F11" s="64" t="n">
         <v>46339</v>
       </c>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I9" s="61" t="n"/>
-    </row>
-    <row r="10" ht="28.05" customHeight="1" s="19">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="G11" s="54" t="n"/>
+      <c r="H11" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I11" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J11" s="56" t="inlineStr">
+        <is>
+          <t>1. Target-State vs. Current-State Dispute Process Gap Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" s="19">
+      <c r="A12" s="53" t="n"/>
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>Conduct review sessions with Loni B. and Pattie L.</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
         <is>
           <t>Loni B. / Pattie L.</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E12" s="64" t="n">
         <v>46314</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F12" s="64" t="n">
         <v>46339</v>
       </c>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I10" s="61" t="n"/>
-    </row>
-    <row r="11" ht="28.05" customHeight="1" s="19">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Incorporate feedback &amp; finalize process maps and operational controls</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="G12" s="54" t="n"/>
+      <c r="H12" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I12" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J12" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1" s="19">
+      <c r="A13" s="59" t="n"/>
+      <c r="B13" s="56" t="inlineStr">
+        <is>
+          <t>Incorporate feedback &amp; finalize process maps and operational controls, including first-party dispute monitoring &amp; review process</t>
+        </is>
+      </c>
+      <c r="C13" s="56" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D13" s="56" t="inlineStr">
         <is>
           <t>Loni B. / Pattie L.</t>
         </is>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E13" s="65" t="n">
         <v>46342</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F13" s="65" t="n">
         <v>46346</v>
       </c>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I11" s="62" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="n"/>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="G13" s="56" t="n"/>
+      <c r="H13" s="59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I13" s="59" t="inlineStr">
+        <is>
+          <t>FD-06, FD-07, FD-08, FD-10</t>
+        </is>
+      </c>
+      <c r="J13" s="56" t="inlineStr">
+        <is>
+          <t>2. Finalized Target-State Dispute Management Process, SOPs &amp; Process Maps (incl. first-party dispute monitoring &amp; review)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1" s="19">
+      <c r="A14" s="59" t="n"/>
+      <c r="B14" s="56" t="inlineStr">
         <is>
           <t>Completion of Dispute Resolution Transformation Activities</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Milestone</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n">
+      <c r="C14" s="56" t="n"/>
+      <c r="D14" s="56" t="n"/>
+      <c r="E14" s="59" t="n"/>
+      <c r="F14" s="65" t="n">
         <v>46346</v>
       </c>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="8" t="n"/>
+      <c r="G14" s="56" t="n"/>
+      <c r="H14" s="59" t="n"/>
+      <c r="I14" s="59" t="n"/>
+      <c r="J14" s="56" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I6:I11"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3292,17 +3717,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="19" min="1" max="1"/>
     <col width="52" customWidth="1" style="19" min="2" max="2"/>
     <col width="12" customWidth="1" style="19" min="3" max="3"/>
-    <col width="30" customWidth="1" style="19" min="4" max="4"/>
+    <col width="12.5" customWidth="1" style="19" min="4" max="4"/>
     <col width="13" customWidth="1" style="19" min="5" max="6"/>
+    <col width="13" customWidth="1" style="19" min="6" max="6"/>
     <col width="22" customWidth="1" style="19" min="7" max="7"/>
     <col width="12" customWidth="1" style="19" min="8" max="8"/>
-    <col width="68.77734375" customWidth="1" style="19" min="9" max="9"/>
+    <col width="13" customWidth="1" style="19" min="9" max="9"/>
+    <col width="68" customWidth="1" style="19" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.05" customHeight="1" s="19">
@@ -3316,485 +3743,652 @@
       <c r="A2" s="18" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="A4" s="66" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B4" s="1" t="inlineStr">
-        <is>
-          <t>Activity / Sub-Activity</t>
-        </is>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="D4" s="1" t="inlineStr">
-        <is>
-          <t>Point of Contact</t>
-        </is>
-      </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="B4" s="66" t="inlineStr">
+        <is>
+          <t>SOW Activity / Sub-Activity</t>
+        </is>
+      </c>
+      <c r="C4" s="66" t="inlineStr">
+        <is>
+          <t>Deloitte Owner</t>
+        </is>
+      </c>
+      <c r="D4" s="66" t="inlineStr">
+        <is>
+          <t>Beem Point of Contact</t>
+        </is>
+      </c>
+      <c r="E4" s="66" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F4" s="66" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G4" s="66" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H4" s="66" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="I4" s="67" t="inlineStr">
+        <is>
+          <t>Req ID</t>
+        </is>
+      </c>
+      <c r="J4" s="68" t="inlineStr">
         <is>
           <t>Deliverables</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="19">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="48" t="n">
         <v>11</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Enhance Existing TPRM Process</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>Review and enhance existing third-party risk management processes to incorporate Visa Debit and BIN Sponsorship requirements, ensuring vendor oversight activities align with applicable regulatory, network, and contractual obligations.</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="63" t="n">
         <v>46321</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="F5" s="63" t="n">
         <v>46339</v>
       </c>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I5" s="22" t="inlineStr">
-        <is>
-          <t>a. Enhanced TPRM Process &amp; Procedures (Visa Debit &amp; BIN Sponsorship requirements)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="28.05" customHeight="1" s="19">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Collect and assess current process against Visa Debit &amp; BIN Sponsorship requirements current TPRM policies &amp; processes</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="G5" s="49" t="n"/>
+      <c r="H5" s="48" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I5" s="52" t="n"/>
+      <c r="J5" s="57" t="n"/>
+    </row>
+    <row r="6" ht="24" customHeight="1" s="19">
+      <c r="A6" s="53" t="n"/>
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>Collect and assess current TPRM policies &amp; processes against Visa Debit &amp; BIN Sponsorship requirements</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D6" s="54" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="64" t="n">
         <v>46321</v>
       </c>
-      <c r="F6" s="7" t="n">
+      <c r="F6" s="64" t="n">
         <v>46325</v>
       </c>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I6" s="25" t="inlineStr">
-        <is>
-          <t>Review and and enhance existing third-party risk management processes to incorporate Visa Debit and BIN Sponsorship requirements, ensuring vendor oversight activities align with applicable regulatory, network, and contractual obligations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="28.05" customHeight="1" s="19">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Draft enhanced TPRM process &amp; controls</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="G6" s="54" t="n"/>
+      <c r="H6" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I6" s="42" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J6" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1" s="19">
+      <c r="A7" s="53" t="n"/>
+      <c r="B7" s="54" t="inlineStr">
+        <is>
+          <t>Draft enhanced TPA contracting review process &amp; controls (Visa-mandated clauses)</t>
+        </is>
+      </c>
+      <c r="C7" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D7" s="54" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="64" t="n">
         <v>46328</v>
       </c>
-      <c r="F7" s="7" t="n">
+      <c r="F7" s="64" t="n">
+        <v>46330</v>
+      </c>
+      <c r="G7" s="54" t="n"/>
+      <c r="H7" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I7" s="59" t="inlineStr">
+        <is>
+          <t>TPA-01</t>
+        </is>
+      </c>
+      <c r="J7" s="56" t="inlineStr">
+        <is>
+          <t>1. Enhanced TPA Contracting Review Process (Visa-mandated clause checklist)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" s="19">
+      <c r="A8" s="53" t="n"/>
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t>Draft enhanced TPA due diligence process &amp; controls</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D8" s="54" t="inlineStr">
+        <is>
+          <t>Akinwale A.</t>
+        </is>
+      </c>
+      <c r="E8" s="64" t="n">
+        <v>46330</v>
+      </c>
+      <c r="F8" s="64" t="n">
         <v>46332</v>
       </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I7" s="61" t="n"/>
-    </row>
-    <row r="8" ht="28.05" customHeight="1" s="19">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="G8" s="54" t="n"/>
+      <c r="H8" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I8" s="59" t="inlineStr">
+        <is>
+          <t>TPA-02</t>
+        </is>
+      </c>
+      <c r="J8" s="56" t="inlineStr">
+        <is>
+          <t>2. Enhanced TPA Due Diligence Process &amp; Controls</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1" s="19">
+      <c r="A9" s="53" t="n"/>
+      <c r="B9" s="54" t="inlineStr">
+        <is>
+          <t>Draft TPA relationship change / Sponsor Bank notification process</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>Akinwale A.</t>
+        </is>
+      </c>
+      <c r="E9" s="64" t="n">
+        <v>46332</v>
+      </c>
+      <c r="F9" s="64" t="n">
+        <v>46335</v>
+      </c>
+      <c r="G9" s="54" t="n"/>
+      <c r="H9" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I9" s="42" t="inlineStr">
+        <is>
+          <t>TPA-03</t>
+        </is>
+      </c>
+      <c r="J9" s="56" t="inlineStr">
+        <is>
+          <t>3. TPA Relationship Change &amp; Sponsor Bank Notification Process</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1" s="19">
+      <c r="A10" s="53" t="n"/>
+      <c r="B10" s="54" t="inlineStr">
         <is>
           <t>Review &amp; finalize with Akinwale A.</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D10" s="54" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E10" s="64" t="n">
         <v>46335</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F10" s="64" t="n">
         <v>46339</v>
       </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I8" s="62" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1" s="19">
-      <c r="A9" s="2" t="n">
+      <c r="G10" s="54" t="n"/>
+      <c r="H10" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I10" s="42" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J10" s="56" t="n"/>
+    </row>
+    <row r="11" ht="30" customHeight="1" s="19">
+      <c r="A11" s="48" t="n">
         <v>12</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Establish ICICI Attestation Process</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="B11" s="49" t="inlineStr">
+        <is>
+          <t>Establish process to submit annual Attestation of Compliance to ICICI Bank.</t>
+        </is>
+      </c>
+      <c r="C11" s="49" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D11" s="49" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E11" s="63" t="n">
         <v>46342</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="F11" s="63" t="n">
         <v>46353</v>
       </c>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I9" s="22" t="inlineStr">
-        <is>
-          <t>b. Annual ICICI Attestation of Compliance Submission Process</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="28.05" customHeight="1" s="19">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="G11" s="49" t="n"/>
+      <c r="H11" s="48" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I11" s="58" t="n"/>
+      <c r="J11" s="57" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1" s="19">
+      <c r="A12" s="53" t="n"/>
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>Collect and review excerpt of ICICI contract (attestation requirements, templates, submission guidance)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D12" s="54" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E12" s="64" t="n">
         <v>46342</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F12" s="64" t="n">
         <v>46344</v>
       </c>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I10" s="25" t="inlineStr">
-        <is>
-          <t>Establish process to submit annual Attestation of Compliance to ICICI Bank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28.05" customHeight="1" s="19">
-      <c r="A11" s="5" t="n"/>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Draft annual Attestation of Compliance submission process</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="G12" s="54" t="n"/>
+      <c r="H12" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I12" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J12" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1" s="19">
+      <c r="A13" s="53" t="n"/>
+      <c r="B13" s="54" t="inlineStr">
+        <is>
+          <t>Draft annual ICICI Attestation of Compliance submission process</t>
+        </is>
+      </c>
+      <c r="C13" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D13" s="54" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E13" s="64" t="n">
         <v>46345</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F13" s="64" t="n">
         <v>46349</v>
       </c>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I11" s="61" t="n"/>
-    </row>
-    <row r="12" ht="28.05" customHeight="1" s="19">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="G13" s="54" t="n"/>
+      <c r="H13" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I13" s="42" t="inlineStr">
+        <is>
+          <t>OS-04</t>
+        </is>
+      </c>
+      <c r="J13" s="56" t="inlineStr">
+        <is>
+          <t>1. Annual ICICI Attestation of Compliance Submission Process</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1" s="19">
+      <c r="A14" s="53" t="n"/>
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t>Review &amp; finalize with Akinwale A. / Pattie L.</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D14" s="54" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E14" s="64" t="n">
         <v>46350</v>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F14" s="64" t="n">
         <v>46353</v>
       </c>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I12" s="62" t="n"/>
-    </row>
-    <row r="13" ht="45" customHeight="1" s="19">
-      <c r="A13" s="2" t="n">
+      <c r="G14" s="54" t="n"/>
+      <c r="H14" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I14" s="42" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J14" s="56" t="n"/>
+    </row>
+    <row r="15" ht="30" customHeight="1" s="19">
+      <c r="A15" s="48" t="n">
         <v>13</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Build Centralized Artifact Repository</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>Design and implement a centralized artifact repository and communication framework to support Visa Debit oversight activities, including storage and management of policies, procedures, reporting artifacts, compliance evidence, governance documentation, issue logs, and correspondence with regulators, Visa, and 3rd parties.</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D15" s="49" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E15" s="63" t="n">
         <v>46356</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="F15" s="63" t="n">
         <v>46367</v>
       </c>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I13" s="22" t="inlineStr">
-        <is>
-          <t>a. Centralized Artifact Repository (policies, procedures, reporting artifacts, compliance evidence, governance docs, issue logs)
-b. Oversight Communication Framework (regulator, Visa &amp; third-party correspondence)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="28.05" customHeight="1" s="19">
-      <c r="A14" s="5" t="n"/>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Design repository structure &amp; communication framework - Working Sessions with Akinwale to align on structure</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="G15" s="49" t="n"/>
+      <c r="H15" s="48" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I15" s="58" t="n"/>
+      <c r="J15" s="57" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1" s="19">
+      <c r="A16" s="53" t="n"/>
+      <c r="B16" s="54" t="inlineStr">
+        <is>
+          <t>Design repository structure &amp; communication framework - working session with Akinwale to align on structure</t>
+        </is>
+      </c>
+      <c r="C16" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D16" s="54" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E16" s="64" t="n">
         <v>46356</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F16" s="64" t="n">
         <v>46360</v>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="G16" s="54" t="inlineStr">
         <is>
           <t>N/A - no doc needed</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I14" s="25" t="inlineStr">
-        <is>
-          <t>Design and implement a centralized artifact repository and communication framework to support Visa Debit oversight activities, including storage and management of policies, procedures, reporting artifacts, compliance evidence, governance documentation, issue logs, and correspondence with regulators, Visa, and 3rd parties.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="28.05" customHeight="1" s="19">
-      <c r="A15" s="5" t="n"/>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Configure &amp; populate repository (policies, procedures, reporting artifacts, compliance evidence, governance docs, issue logs)</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
+      <c r="H16" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I16" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J16" s="56" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1" s="19">
+      <c r="A17" s="53" t="n"/>
+      <c r="B17" s="54" t="inlineStr">
+        <is>
+          <t>Configure &amp; populate repository (policies, procedures, reporting artifacts, compliance evidence, governance docs, issue logs) to support ongoing compliance monitoring</t>
+        </is>
+      </c>
+      <c r="C17" s="54" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D17" s="54" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E17" s="64" t="n">
         <v>46363</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F17" s="64" t="n">
+        <v>46365</v>
+      </c>
+      <c r="G17" s="54" t="n"/>
+      <c r="H17" s="53" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I17" s="59" t="inlineStr">
+        <is>
+          <t>OS-01, OS-03</t>
+        </is>
+      </c>
+      <c r="J17" s="56" t="inlineStr">
+        <is>
+          <t>1. Centralized Artifact Repository (policies, procedures, reporting artifacts, compliance evidence, governance docs, issue logs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1" s="19">
+      <c r="A18" s="59" t="n"/>
+      <c r="B18" s="56" t="inlineStr">
+        <is>
+          <t>Build communication framework for regulator / Visa / third-party correspondence</t>
+        </is>
+      </c>
+      <c r="C18" s="56" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D18" s="56" t="inlineStr">
+        <is>
+          <t>Akinwale A.</t>
+        </is>
+      </c>
+      <c r="E18" s="65" t="n">
+        <v>46365</v>
+      </c>
+      <c r="F18" s="65" t="n">
         <v>46367</v>
       </c>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I15" s="61" t="n"/>
-    </row>
-    <row r="16" ht="28.05" customHeight="1" s="19">
-      <c r="A16" s="5" t="n"/>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="G18" s="56" t="n"/>
+      <c r="H18" s="59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I18" s="59" t="inlineStr">
+        <is>
+          <t>OS-02</t>
+        </is>
+      </c>
+      <c r="J18" s="56" t="inlineStr">
+        <is>
+          <t>2. Oversight Communication Framework (regulator, Visa &amp; third-party correspondence)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1" s="19">
+      <c r="A19" s="59" t="n"/>
+      <c r="B19" s="56" t="inlineStr">
         <is>
           <t>Review &amp; hand over to Beem</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Sub-Activity</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="C19" s="56" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="D19" s="56" t="inlineStr">
         <is>
           <t>Akinwale A.</t>
         </is>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E19" s="65" t="n">
         <v>46363</v>
       </c>
-      <c r="F16" s="7" t="n">
+      <c r="F19" s="65" t="n">
         <v>46367</v>
       </c>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="I16" s="62" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="n"/>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="G19" s="56" t="n"/>
+      <c r="H19" s="59" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="I19" s="59" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J19" s="56" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1" s="19">
+      <c r="A20" s="59" t="n"/>
+      <c r="B20" s="56" t="inlineStr">
         <is>
           <t>Completion of TPRM &amp; Oversight Transformation Activities</t>
         </is>
       </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>Milestone</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="n">
+      <c r="C20" s="56" t="n"/>
+      <c r="D20" s="56" t="n"/>
+      <c r="E20" s="59" t="n"/>
+      <c r="F20" s="65" t="n">
         <v>46367</v>
       </c>
-      <c r="G17" s="9" t="n"/>
-      <c r="H17" s="8" t="n"/>
+      <c r="G20" s="56" t="n"/>
+      <c r="H20" s="59" t="n"/>
+      <c r="I20" s="59" t="n"/>
+      <c r="J20" s="56" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="I6:I8"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="I10:I12"/>
-    <mergeCell ref="I14:I16"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix Process/System Req ID mixing in generated activities
Following the pattern in the manager's Activity #1 (which cites only
Functional (Process) requirements for its process/SOP deliverables),
removed System-type Req IDs that had been mixed into process-oriented
deliverables in Fraud #5, AML #7/#8, and Dispute Resolution #9.
System-type reqs remain correctly cited only where the deliverable
itself is a system requirements spec (Fraud #2 DataVisor).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Msiz5p6hoKmmUHZyLJTkqb
</commit_message>
<xml_diff>
--- a/Beem Visa Debit Transformation Phase Project Plan v3.xlsx
+++ b/Beem Visa Debit Transformation Phase Project Plan v3.xlsx
@@ -2213,7 +2213,7 @@
       </c>
       <c r="I34" s="59" t="inlineStr">
         <is>
-          <t>FD-19, FD-20, FD-21</t>
+          <t>FD-19, FD-20</t>
         </is>
       </c>
       <c r="J34" s="56" t="inlineStr">
@@ -2911,7 +2911,7 @@
       </c>
       <c r="I16" s="42" t="inlineStr">
         <is>
-          <t>AML-02</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J16" s="56" t="inlineStr">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="I17" s="42" t="inlineStr">
         <is>
-          <t>AML-02, AML-11</t>
+          <t>AML-11</t>
         </is>
       </c>
       <c r="J17" s="56" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="I23" s="59" t="inlineStr">
         <is>
-          <t>AML-09, AML-10</t>
+          <t>AML-09</t>
         </is>
       </c>
       <c r="J23" s="56" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="I6" s="42" t="inlineStr">
         <is>
-          <t>FD-05, FD-06</t>
+          <t>FD-06</t>
         </is>
       </c>
       <c r="J6" s="56" t="inlineStr">

</xml_diff>

<commit_message>
Enrich deliverable descriptions with requirement-derived detail
Matches Activity #1's depth: each deliverable's parenthetical now
pulls specific mechanics from its mapped requirement's Acceptance
Criteria text (e.g., specific metrics, disposition options, timeframes,
system behaviors) rather than a generic title.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Msiz5p6hoKmmUHZyLJTkqb
</commit_message>
<xml_diff>
--- a/Beem Visa Debit Transformation Phase Project Plan v3.xlsx
+++ b/Beem Visa Debit Transformation Phase Project Plan v3.xlsx
@@ -1608,7 +1608,7 @@
       </c>
       <c r="J18" s="56" t="inlineStr">
         <is>
-          <t>1. DataVisor Data Integration Architecture &amp; Requirements</t>
+          <t>1. DataVisor Data Integration Architecture &amp; Requirements (transaction ingestion pipeline, fraud rule/model configuration, data sourcing from DNA/Everlink)</t>
         </is>
       </c>
     </row>
@@ -1648,7 +1648,7 @@
       </c>
       <c r="J19" s="56" t="inlineStr">
         <is>
-          <t>2. DataVisor Fraud Monitoring Use Cases &amp; Detection/Alerting Rules</t>
+          <t>2. DataVisor Fraud Monitoring Use Cases &amp; Detection/Alerting Rules (rule/model-triggered alert generation, case management functionality, automatic card-block request to core banking system upon suspected/confirmed fraud)</t>
         </is>
       </c>
     </row>
@@ -1688,7 +1688,7 @@
       </c>
       <c r="J20" s="43" t="inlineStr">
         <is>
-          <t>3. DataVisor Governance &amp; Oversight Considerations</t>
+          <t>3. DataVisor Governance &amp; Oversight Considerations (rule/model change control, access management, oversight cadence)</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="J30" s="56" t="inlineStr">
         <is>
-          <t>1. Analytics-Driven Fraud Detection Process (authentication failure pattern analysis methodology)</t>
+          <t>1. Analytics-Driven Fraud Detection Process (ongoing authentication failure pattern &amp; root-cause analysis methodology, rule-tuning opportunity assessment, findings/recommendation documentation)</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="J34" s="56" t="inlineStr">
         <is>
-          <t>1. Internal Fraud Reporting Framework (fraud loss reporting, VIMP threshold monitoring, management reporting)</t>
+          <t>1. Internal Fraud Reporting Framework (fraud/dispute volume &amp; threshold monitoring with escalation triggers; management reporting metrics — Net/Gross Fraud Losses, Fraud-to-Sales Ratios (CP/CNP), Fraud Decline Rate, Dispute Volumes/Ratios, alert volume &amp; aging, penetration rate)</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="J35" s="56" t="inlineStr">
         <is>
-          <t>2. Visa Fraud Reporting System (FRS) Submission Process</t>
+          <t>2. Visa Fraud Reporting System (FRS) Submission Process (confirmed case data preparation, submission within Visa reporting timeframe, submission date/status documentation)</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="J36" s="56" t="inlineStr">
         <is>
-          <t>3. ICICI Sponsor Bank Fraud Reporting Process</t>
+          <t>3. ICICI Sponsor Bank Fraud Reporting Process (suspected/confirmed case reporting within ICICI-established timeframe, submission date/status documentation)</t>
         </is>
       </c>
     </row>
@@ -2597,12 +2597,12 @@
       </c>
       <c r="I8" s="59" t="inlineStr">
         <is>
-          <t>AML-01</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J8" s="56" t="inlineStr">
         <is>
-          <t>1. Enhanced AML Policies, Procedures &amp; Governance Controls (Visa Debit)</t>
+          <t>1. Enhanced AML Policies, Procedures &amp; Governance Controls (Visa Debit) (how Visa Debit falls within AML/ATF policy scope, governance roles &amp; accountability, program obligations and expectations)</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="J9" s="56" t="inlineStr">
         <is>
-          <t>2. Sanctions Screening Process &amp; Requirements (OFAC SDN screening, true-match card/account disablement)</t>
+          <t>2. Sanctions Screening Process &amp; Requirements (OFAC SDN screening at onboarding/issuance &amp; ongoing basis; true-match access disablement in core banking system, Visa/regulatory notification, and remediation documentation)</t>
         </is>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
       </c>
       <c r="J10" s="56" t="inlineStr">
         <is>
-          <t>3. AML Investigation &amp; Case Management Process</t>
+          <t>3. AML Investigation &amp; Case Management Process (alert investigation and disposition — cleared, escalated, STR filed — with documented outcome)</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="J11" s="56" t="inlineStr">
         <is>
-          <t>4. AML Regulatory &amp; Sponsor Bank Reporting Requirements (FINTRAC STR/EFT/LCT, ICICI)</t>
+          <t>4. AML Regulatory &amp; Sponsor Bank Reporting Requirements (FINTRAC STR/EFT/LCT reportability assessment &amp; submission within regulatory timeframe with record retention; ICICI Sponsor Bank reporting with submission date/status documentation)</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="J17" s="56" t="inlineStr">
         <is>
-          <t>2. AML Monitoring Rules &amp; Alert Scenarios</t>
+          <t>2. AML Monitoring Rules &amp; Alert Scenarios (rule creation/maintenance approach with documented, tested, and approved change process prior to production implementation)</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="J18" s="56" t="inlineStr">
         <is>
-          <t>3. AML Monitoring Rules Testing &amp; Validation Summary</t>
+          <t>3. AML Monitoring Rules Testing &amp; Validation Summary (validates rule deployment against defined variables/syntax/logic without exceeding system performance thresholds)</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="J19" s="56" t="inlineStr">
         <is>
-          <t>4. AML Monitoring Production Readiness &amp; Operationalization Checklist</t>
+          <t>4. AML Monitoring Production Readiness &amp; Operationalization Checklist (production deployment, modification, and deactivation of rules within system performance thresholds)</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
       </c>
       <c r="J23" s="56" t="inlineStr">
         <is>
-          <t>1. Internal AML Reporting Framework (operational &amp; analytics performance reports)</t>
+          <t>1. Internal AML Reporting Framework (STR filing root-cause/driver breakdown, alert-to-STR conversion rate, open case aging, sanctions true-match rate, manually generated UAR count, member risk-rating migration rate, demarketing/deservicing rate)</t>
         </is>
       </c>
     </row>
@@ -3406,7 +3406,7 @@
       </c>
       <c r="J6" s="56" t="inlineStr">
         <is>
-          <t>1. Target-State Dispute Intake &amp; Fraud/Non-Fraud Determination Process</t>
+          <t>1. Target-State Dispute Intake &amp; Fraud/Non-Fraud Determination Process (transaction activity, cardholder history, authentication results &amp; evidence review; documented determination, rationale, and resulting actions within Visa timeframes)</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="J7" s="56" t="inlineStr">
         <is>
-          <t>2. Target-State Provisional Credit, Chargeback (Central 1) &amp; Visa Dispute Processing Flow</t>
+          <t>2. Target-State Provisional Credit, Chargeback (Central 1) &amp; Visa Dispute Processing Flow (eligible dispute preparation with required information/evidence, submission to Central 1 for VROL within Visa's required timeframe)</t>
         </is>
       </c>
     </row>
@@ -3486,7 +3486,7 @@
       </c>
       <c r="J8" s="56" t="inlineStr">
         <is>
-          <t>3. Target-State Funds Recovery Process &amp; Supporting Procedures/Process Maps</t>
+          <t>3. Target-State Funds Recovery Process &amp; Supporting Procedures/Process Maps (dispute lifecycle management across response review, pre-arbitration, arbitration, compliance proceedings, recovery &amp; closure, with documented outcomes within Visa timeframes)</t>
         </is>
       </c>
     </row>
@@ -3680,7 +3680,7 @@
       </c>
       <c r="J13" s="56" t="inlineStr">
         <is>
-          <t>2. Finalized Target-State Dispute Management Process, SOPs &amp; Process Maps (incl. first-party dispute monitoring &amp; review)</t>
+          <t>2. Finalized Target-State Dispute Management Process, SOPs &amp; Process Maps (incl. 5+ dispute/12-month first-party fraud monitoring trigger, cardholder history/behavior review, and escalation criteria)</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="J7" s="56" t="inlineStr">
         <is>
-          <t>1. Enhanced TPA Contracting Review Process (Visa-mandated clause checklist)</t>
+          <t>1. Enhanced TPA Contracting Review Process (Visa-mandated clause checklist — policies, procedures, service levels, performance standards, dispute handling, fraud reporting, settlement workflows, roles/responsibilities, security obligations, audit rights, incident management — with pre-execution amendment tracking)</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3944,7 @@
       </c>
       <c r="J8" s="56" t="inlineStr">
         <is>
-          <t>2. Enhanced TPA Due Diligence Process &amp; Controls</t>
+          <t>2. Enhanced TPA Due Diligence Process &amp; Controls (initial &amp; ongoing due diligence file review with gap identification, escalation, and remediation tracking through closure)</t>
         </is>
       </c>
     </row>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="J9" s="56" t="inlineStr">
         <is>
-          <t>3. TPA Relationship Change &amp; Sponsor Bank Notification Process</t>
+          <t>3. TPA Relationship Change &amp; Sponsor Bank Notification Process (ownership change/contract termination notification within internal timeframe to meet Visa's 5-business-day requirement, with documented change details, notification date, recipient &amp; status)</t>
         </is>
       </c>
     </row>
@@ -4134,7 +4134,7 @@
       </c>
       <c r="J13" s="56" t="inlineStr">
         <is>
-          <t>1. Annual ICICI Attestation of Compliance Submission Process</t>
+          <t>1. Annual ICICI Attestation of Compliance Submission Process (officer attestation preparation, completion, signature &amp; submission to ICICI before March 31 each year)</t>
         </is>
       </c>
     </row>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="J17" s="56" t="inlineStr">
         <is>
-          <t>1. Centralized Artifact Repository (policies, procedures, reporting artifacts, compliance evidence, governance docs, issue logs)</t>
+          <t>1. Centralized Artifact Repository (policies, procedures, reporting artifacts, compliance evidence, governance docs, issue logs — supporting compliance status tracking, gap remediation, and Visa Rule change tracking through implementation)</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="J18" s="56" t="inlineStr">
         <is>
-          <t>2. Oversight Communication Framework (regulator, Visa &amp; third-party correspondence)</t>
+          <t>2. Oversight Communication Framework (regulator, Visa &amp; third-party correspondence with tracked response timeframes and completion status)</t>
         </is>
       </c>
     </row>

</xml_diff>